<commit_message>
feat: stream XLSX cells to avoid large-file allocation; remove quoting mode 3
- Replace worksheet_range() with worksheet_cells_reader() for XLSX: cells
  are now emitted one row at a time so a declared A1:XFD1048576 sheet no
  longer forces a ~550 GB allocation; add MAX_ROW/MAX_COL bounds check
- Add convert_sheet() dispatcher routing XLSX to streaming and XLS to the
  existing dense Range path; reject Xlsb/Ods formats with a clear error
- Remove --out-quoting mode 3 (csv::QuoteStyle::Never): it can emit
  unquoted delimiters and newlines, producing malformed output
- Fix render_datetime to preserve milliseconds (.500 suffix when non-zero)
- Add 200-byte length cap to sanitize_sheet_name to prevent ENAMETOOLONG
- Expand types fixture with datetime-with-ms and leading-zero string rows
- Add sanitize_sheet_name unit tests (path traversal, dot names, long names)
- Update integration tests: mode-3 rejection, XLSB/ODS rejection, range check

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/types.xlsx
+++ b/tests/fixtures/types.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>type</t>
   </si>
@@ -38,14 +38,24 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>datetime_ms</t>
+  </si>
+  <si>
+    <t>leading_zero</t>
+  </si>
+  <si>
+    <t>007</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss.000"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -76,9 +86,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -373,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -429,6 +440,22 @@
         <v>45306</v>
       </c>
     </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45366.60469328704</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>